<commit_message>
docs: phân công use case theo thành viên
Thêm cột Người phụ trách cho 42 UC và bảng phân công ở sheet Tong hop.
Theo bảng RACI Báo cáo 2 (mục II.4); PN chuyển từ NghiaNV sang DongLV,
HT-06 theo hàng "Khung giao diện, thông báo" (QuangTD).
</commit_message>
<xml_diff>
--- a/docs/SFEMS_Danh-sach-UC-pham-vi-do-an.xlsx
+++ b/docs/SFEMS_Danh-sach-UC-pham-vi-do-an.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -538,6 +538,7 @@
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -554,6 +555,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Người phụ trách theo bảng RACI ở Báo cáo 2 (mục II.4); PN chuyển từ NghiaNV sang DongLV, HT-06 theo hàng "Khung giao diện, thông báo" (QuangTD).</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -583,6 +591,11 @@
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Mã cũ (bản nộp lần 1)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Người phụ trách</t>
         </is>
       </c>
     </row>
@@ -596,7 +609,8 @@
       <c r="C5" s="10" t="n"/>
       <c r="D5" s="10" t="n"/>
       <c r="E5" s="10" t="n"/>
-      <c r="F5" s="11" t="n"/>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="11" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
@@ -627,6 +641,11 @@
           <t>HT-01</t>
         </is>
       </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>DongLV</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
@@ -657,6 +676,11 @@
           <t>HT-02</t>
         </is>
       </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>DongLV</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
@@ -687,6 +711,11 @@
           <t>HT-03</t>
         </is>
       </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>DongLV</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
@@ -717,6 +746,11 @@
           <t>HT-05</t>
         </is>
       </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>DongLV</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
@@ -747,6 +781,11 @@
           <t>HT-07</t>
         </is>
       </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>DongLV</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
@@ -775,6 +814,11 @@
       <c r="F11" s="7" t="inlineStr">
         <is>
           <t>HT-10</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>QuangTD</t>
         </is>
       </c>
     </row>
@@ -788,7 +832,8 @@
       <c r="C12" s="10" t="n"/>
       <c r="D12" s="10" t="n"/>
       <c r="E12" s="10" t="n"/>
-      <c r="F12" s="11" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
@@ -819,6 +864,11 @@
           <t>DM-01</t>
         </is>
       </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
@@ -849,6 +899,11 @@
           <t>DM-02</t>
         </is>
       </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
@@ -879,6 +934,11 @@
           <t>DM-03</t>
         </is>
       </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
@@ -907,6 +967,11 @@
       <c r="F16" s="7" t="inlineStr">
         <is>
           <t>DM-04</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
         </is>
       </c>
     </row>
@@ -920,7 +985,8 @@
       <c r="C17" s="10" t="n"/>
       <c r="D17" s="10" t="n"/>
       <c r="E17" s="10" t="n"/>
-      <c r="F17" s="11" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
@@ -951,6 +1017,11 @@
           <t>TC-01</t>
         </is>
       </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>HoangPND</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
@@ -979,6 +1050,11 @@
       <c r="F19" s="7" t="inlineStr">
         <is>
           <t>CS-03</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>HoangPND</t>
         </is>
       </c>
     </row>
@@ -992,7 +1068,8 @@
       <c r="C20" s="10" t="n"/>
       <c r="D20" s="10" t="n"/>
       <c r="E20" s="10" t="n"/>
-      <c r="F20" s="11" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
@@ -1023,6 +1100,11 @@
           <t>TS-01</t>
         </is>
       </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>NghiaNV</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
@@ -1053,6 +1135,11 @@
           <t>TS-02</t>
         </is>
       </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>NghiaNV</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
@@ -1083,6 +1170,11 @@
           <t>TS-05</t>
         </is>
       </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>NghiaNV</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
@@ -1113,6 +1205,11 @@
           <t>TS-06</t>
         </is>
       </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>NghiaNV</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
@@ -1143,6 +1240,11 @@
           <t>TS-07</t>
         </is>
       </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>NghiaNV</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
@@ -1173,6 +1275,11 @@
           <t>TS-08</t>
         </is>
       </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>NghiaNV</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
@@ -1201,6 +1308,11 @@
       <c r="F27" s="7" t="inlineStr">
         <is>
           <t>TS-09</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>NghiaNV</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1326,8 @@
       <c r="C28" s="10" t="n"/>
       <c r="D28" s="10" t="n"/>
       <c r="E28" s="10" t="n"/>
-      <c r="F28" s="11" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
@@ -1245,6 +1358,11 @@
           <t>NC-01</t>
         </is>
       </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>HoangPND</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
@@ -1275,6 +1393,11 @@
           <t>NC-02 + NC-03</t>
         </is>
       </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>HoangPND</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
@@ -1305,6 +1428,11 @@
           <t>NC-04</t>
         </is>
       </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>HoangPND</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
@@ -1335,6 +1463,11 @@
           <t>NC-05</t>
         </is>
       </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>HoangPND</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
@@ -1365,6 +1498,11 @@
           <t>NC-06</t>
         </is>
       </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>HoangPND</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
@@ -1395,6 +1533,11 @@
           <t>NC-07</t>
         </is>
       </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>HoangPND</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
@@ -1423,6 +1566,11 @@
       <c r="F35" s="7" t="inlineStr">
         <is>
           <t>NC-09</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>HoangPND</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1584,8 @@
       <c r="C36" s="10" t="n"/>
       <c r="D36" s="10" t="n"/>
       <c r="E36" s="10" t="n"/>
-      <c r="F36" s="11" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
@@ -1467,6 +1616,11 @@
           <t>PN-01 + PN-02 + PN-03</t>
         </is>
       </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>DongLV</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
@@ -1497,6 +1651,11 @@
           <t>PN-04</t>
         </is>
       </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>DongLV</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
@@ -1525,6 +1684,11 @@
       <c r="F39" s="7" t="inlineStr">
         <is>
           <t>PN-05</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>DongLV</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1702,8 @@
       <c r="C40" s="10" t="n"/>
       <c r="D40" s="10" t="n"/>
       <c r="E40" s="10" t="n"/>
-      <c r="F40" s="11" t="n"/>
+      <c r="F40" s="10" t="n"/>
+      <c r="G40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
@@ -1569,6 +1734,11 @@
           <t>KK-01</t>
         </is>
       </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
@@ -1599,6 +1769,11 @@
           <t>KK-02</t>
         </is>
       </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
@@ -1629,6 +1804,11 @@
           <t>KK-03</t>
         </is>
       </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
@@ -1659,6 +1839,11 @@
           <t>KK-04 + KK-05</t>
         </is>
       </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
@@ -1689,6 +1874,11 @@
           <t>KK-06</t>
         </is>
       </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
@@ -1719,6 +1909,11 @@
           <t>KK-07</t>
         </is>
       </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
@@ -1747,6 +1942,11 @@
       <c r="F47" s="7" t="inlineStr">
         <is>
           <t>KK-08</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>TuTN</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1960,8 @@
       <c r="C48" s="10" t="n"/>
       <c r="D48" s="10" t="n"/>
       <c r="E48" s="10" t="n"/>
-      <c r="F48" s="11" t="n"/>
+      <c r="F48" s="10" t="n"/>
+      <c r="G48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n">
@@ -1791,6 +1992,11 @@
           <t>BC-01</t>
         </is>
       </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>QuangTD</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
@@ -1821,6 +2027,11 @@
           <t>BC-02 (tách)</t>
         </is>
       </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>QuangTD</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n">
@@ -1851,6 +2062,11 @@
           <t>BC-02 (tách)</t>
         </is>
       </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>QuangTD</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
@@ -1881,6 +2097,11 @@
           <t>BC-02 (tách) + NC-08</t>
         </is>
       </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>QuangTD</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n">
@@ -1911,6 +2132,11 @@
           <t>BC-02 (tách)</t>
         </is>
       </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>QuangTD</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n">
@@ -1941,21 +2167,29 @@
           <t>BC-04</t>
         </is>
       </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>QuangTD</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="A48:F48"/>
-    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A28:G28"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="E5:E54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"S,M,C"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G5:G54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"DongLV,TuTN,HoangPND,NghiaNV,QuangTD"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1968,12 +2202,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2084,6 +2319,161 @@
       </c>
       <c r="B10" s="6">
         <f>IF(B7&gt;=B8,"Đạt","Chưa đạt")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Phân công theo thành viên</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Thành viên</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Số UC</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Từ Medium trở lên</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Hạng mục</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Lưu Văn Đông (DongLV)</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
+        <f>COUNTIF('Danh sach UC'!$G$6:$G$54,"DongLV")</f>
+        <v/>
+      </c>
+      <c r="C14" s="6">
+        <f>COUNTIFS('Danh sach UC'!$G$6:$G$54,"DongLV",'Danh sach UC'!$E$6:$E$54,"M")+COUNTIFS('Danh sach UC'!$G$6:$G$54,"DongLV",'Danh sach UC'!$E$6:$E$54,"C")</f>
+        <v/>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>HT (trừ HT-06); PN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Trần Ngọc Tú (TuTN)</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
+        <f>COUNTIF('Danh sach UC'!$G$6:$G$54,"TuTN")</f>
+        <v/>
+      </c>
+      <c r="C15" s="6">
+        <f>COUNTIFS('Danh sach UC'!$G$6:$G$54,"TuTN",'Danh sach UC'!$E$6:$E$54,"M")+COUNTIFS('Danh sach UC'!$G$6:$G$54,"TuTN",'Danh sach UC'!$E$6:$E$54,"C")</f>
+        <v/>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>DM; KK</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Phạm Nguyễn Duy Hoàng (HoangPND)</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>COUNTIF('Danh sach UC'!$G$6:$G$54,"HoangPND")</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>COUNTIFS('Danh sach UC'!$G$6:$G$54,"HoangPND",'Danh sach UC'!$E$6:$E$54,"M")+COUNTIFS('Danh sach UC'!$G$6:$G$54,"HoangPND",'Danh sach UC'!$E$6:$E$54,"C")</f>
+        <v/>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>TC; NC</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Nguyễn Vũ Nghĩa (NghiaNV)</t>
+        </is>
+      </c>
+      <c r="B17" s="6">
+        <f>COUNTIF('Danh sach UC'!$G$6:$G$54,"NghiaNV")</f>
+        <v/>
+      </c>
+      <c r="C17" s="6">
+        <f>COUNTIFS('Danh sach UC'!$G$6:$G$54,"NghiaNV",'Danh sach UC'!$E$6:$E$54,"M")+COUNTIFS('Danh sach UC'!$G$6:$G$54,"NghiaNV",'Danh sach UC'!$E$6:$E$54,"C")</f>
+        <v/>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Trần Duy Quang (QuangTD)</t>
+        </is>
+      </c>
+      <c r="B18" s="6">
+        <f>COUNTIF('Danh sach UC'!$G$6:$G$54,"QuangTD")</f>
+        <v/>
+      </c>
+      <c r="C18" s="6">
+        <f>COUNTIFS('Danh sach UC'!$G$6:$G$54,"QuangTD",'Danh sach UC'!$E$6:$E$54,"M")+COUNTIFS('Danh sach UC'!$G$6:$G$54,"QuangTD",'Danh sach UC'!$E$6:$E$54,"C")</f>
+        <v/>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>BC; HT-06 (thông báo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Tổng</t>
+        </is>
+      </c>
+      <c r="B19" s="6">
+        <f>SUM(B14:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="6">
+        <f>SUM(C14:C18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Đã phân công đủ?</t>
+        </is>
+      </c>
+      <c r="B20" s="6">
+        <f>IF(B19=B6,"Đủ","Còn UC chưa có người")</f>
         <v/>
       </c>
     </row>

</xml_diff>